<commit_message>
completed testing and some changes
</commit_message>
<xml_diff>
--- a/storage/seeders/questions.xlsx
+++ b/storage/seeders/questions.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="529">
   <si>
     <t>પ્રશ્ન</t>
   </si>
@@ -1126,6 +1126,528 @@
   <si>
     <t>મધુરાષ્ટકમ</t>
   </si>
+  <si>
+    <t>રામેશ્વર ના દર્શન કરતા પહેલા કોને પગે લાગવામાં આવે છે?</t>
+  </si>
+  <si>
+    <t>મલ્લિકાર્જુન</t>
+  </si>
+  <si>
+    <t>હનુમતીશ્વર</t>
+  </si>
+  <si>
+    <t>મહાકાલ</t>
+  </si>
+  <si>
+    <t>ત્રયંબકેશ્વર મહાદેવ ની ત્રીજી આંખ ભક્ત ને માટે શેનું સુચન કરે છે?</t>
+  </si>
+  <si>
+    <t>કર્તવ્યદક્ષતા</t>
+  </si>
+  <si>
+    <t>વાત્સલ્ય</t>
+  </si>
+  <si>
+    <t>બાલીશતા</t>
+  </si>
+  <si>
+    <t>આજે કોઈ ને પોતાનું ગોત્ર ખબર ન હોય તો તેને ક્યાં ગોત્ર નું ઉચ્ચારણ કરવાની શાસ્ત્ર અનુંમતી આપે છે?</t>
+  </si>
+  <si>
+    <t>ગૌતમ</t>
+  </si>
+  <si>
+    <t>વૈદ્યનાથ જ્યોતિર્લીંગ ની સ્થાપના કોને કરી છે?</t>
+  </si>
+  <si>
+    <t>પાર્વતી</t>
+  </si>
+  <si>
+    <t>ગણપતિ</t>
+  </si>
+  <si>
+    <t>રામ</t>
+  </si>
+  <si>
+    <t>વિશ્વ ને સૌપ્રથમ લોકશાહી નો સિધ્ધાંત કોને આપ્યો?</t>
+  </si>
+  <si>
+    <t>જમદગ્નિ</t>
+  </si>
+  <si>
+    <t>કેદારનાથ જ્યોતિર્લીંગ માં નર-નારાયણે શેનું ઉદગાન કર્યું છે?</t>
+  </si>
+  <si>
+    <t>શ્રીસૂક્ત</t>
+  </si>
+  <si>
+    <t>પુરુષસૂક્ત</t>
+  </si>
+  <si>
+    <t>પર્જન્યસૂક્ત</t>
+  </si>
+  <si>
+    <t>મંત્રસુક્ત</t>
+  </si>
+  <si>
+    <t>ગાયમાં ૩૩ કરોડ દેવતા છે એ ભાવનાત્મક વિચાર ક્યાં ઋષી એ આપ્યો?</t>
+  </si>
+  <si>
+    <t>ભરદ્વાજ</t>
+  </si>
+  <si>
+    <t>યાજ્ઞવલ્ક્ય એ સૂર્ય પાસેથી વિચાર અને સરસ્વતી પાસેથી શબ્દ મેળવીને ક્યાં ગ્રંથની રચના કરી?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">અથર્વવેદ </t>
+  </si>
+  <si>
+    <t>સામવેદ</t>
+  </si>
+  <si>
+    <t>શુક્લ યજુર્વેદ</t>
+  </si>
+  <si>
+    <t>કૃષ્ણ યજુર્વેદ</t>
+  </si>
+  <si>
+    <t>ક્યાં જ્યોતિર્લીંગ માં અર્ધનારીનટેશ્વર બનીને ભગવાને દર્શન આપ્યા?</t>
+  </si>
+  <si>
+    <t>નાગેશ્વર</t>
+  </si>
+  <si>
+    <t>મહાકાલેશ્વર</t>
+  </si>
+  <si>
+    <t>વૈદ્યનાથ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">દાદાજીને ટેમ્પલટન એવોર્ડ કઈ સાલમાં મળ્યો હતો? </t>
+  </si>
+  <si>
+    <t>વલભાચાર્યએ આપેલી બાળભક્તિ પાછળના મુખ્ય હેતુ કયા હતા?</t>
+  </si>
+  <si>
+    <t>બાળક પાસે મંગાઈ નહીં</t>
+  </si>
+  <si>
+    <t>બાળક પાસે રડાઈ નહીં</t>
+  </si>
+  <si>
+    <t>બાળક ની મૂર્તિ મનોહર લાગે</t>
+  </si>
+  <si>
+    <t>A અને B બન્ને</t>
+  </si>
+  <si>
+    <t>પૂજનીય દાદાજીએ અર્થશાસ્ત્ર પર આપેલું પુસ્તક કયું?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">શ્રીસુક્તમ </t>
+  </si>
+  <si>
+    <t>સંસ્કૃતિ ચિંતન</t>
+  </si>
+  <si>
+    <t>ભારતીયો નું આદર્શ જીવન</t>
+  </si>
+  <si>
+    <t>તુલસીદલ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">who is father of Indian philosophy? </t>
+  </si>
+  <si>
+    <t>વસિષ્ઠ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">પૂજનીય દાદાજીની પ્રિય રમત </t>
+  </si>
+  <si>
+    <t>હુતુતુ</t>
+  </si>
+  <si>
+    <t>કુસ્તી</t>
+  </si>
+  <si>
+    <t>આટીયા-પાટિયા</t>
+  </si>
+  <si>
+    <t>વોલીબોલ</t>
+  </si>
+  <si>
+    <t>વિદ્યાપ્રેમવર્ધન પરીક્ષામાં પાંચમી પરીક્ષા કઈ છે?</t>
+  </si>
+  <si>
+    <t>પારંગત</t>
+  </si>
+  <si>
+    <t>અનુજ્ઞાતા</t>
+  </si>
+  <si>
+    <t>વિચક્ષણ</t>
+  </si>
+  <si>
+    <t>જ્ઞાતા</t>
+  </si>
+  <si>
+    <t>ભગવાન શ્રીકૃષ્ણના ધનુષ્યનું નામ શું હતું?</t>
+  </si>
+  <si>
+    <t>પાંચજન્ય</t>
+  </si>
+  <si>
+    <t xml:space="preserve">સારંગ </t>
+  </si>
+  <si>
+    <t>પીનાકી</t>
+  </si>
+  <si>
+    <t>કોદંડ</t>
+  </si>
+  <si>
+    <t>માખણ ચોર ની વિચારધારાને પ્રગટ કરતો દાદાજીએ કયો પ્રયોગ આપ્યો?</t>
+  </si>
+  <si>
+    <t>ગોરસ</t>
+  </si>
+  <si>
+    <t>ગૌરીપૂજા</t>
+  </si>
+  <si>
+    <t>એક્વીરા</t>
+  </si>
+  <si>
+    <t>વિદ્યાપીઠ ના બે વર્ષના કોર્સ નું નામ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">આર્યવૃત </t>
+  </si>
+  <si>
+    <t>વિનીત</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ગુરુ દત્તાત્રેય એ કેટલા ગુરુઓ માન્યા હતા? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">પૂજનીય દીદીજીને શિક્ષણ અંગે કયો એવોર્ડ મળ્યો? </t>
+  </si>
+  <si>
+    <t>લોકશિક્ષક એવોર્ડ</t>
+  </si>
+  <si>
+    <t>લોકજાગૃતિ એવોર્ડ</t>
+  </si>
+  <si>
+    <t>લોકસુધારક એવોર્ડ</t>
+  </si>
+  <si>
+    <t>લોકસેવા એવોર્ડ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">પૂજનીય દાદાજીના પ્રવચનોમાંથી મહાભારત પર લખાયેલું પુસ્તક કયું? </t>
+  </si>
+  <si>
+    <t>વ્યાસ વિચાર</t>
+  </si>
+  <si>
+    <t>જીવનતીર્થ</t>
+  </si>
+  <si>
+    <t>પૂજનીય દીદીજી એ પ્રથમ ઉદબોધન ક્યારે કર્યું?</t>
+  </si>
+  <si>
+    <t>ભાવમિલન સમારોહ ૧૯૭૬</t>
+  </si>
+  <si>
+    <t>તીર્થરાજ મિલન ૧૯૮૬</t>
+  </si>
+  <si>
+    <t>સુધાવર્ષ ૨૦૦૧</t>
+  </si>
+  <si>
+    <t>અશીતિ વંદના ૨૦૦૦</t>
+  </si>
+  <si>
+    <t>પ્રથમ મત્સ્યગંધાનુ જલાવરણ કયા વર્ષમાં થયું હતું?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">દાદાજીની પાંચ પેઢીના નામ ક્રમશઃ જણાવો </t>
+  </si>
+  <si>
+    <t>પાંડુરંગપંત – પરશુરામપંત – લક્ષ્મણરાવ – વૈજનાથ –પાંડુરંગશાસ્ત્રી</t>
+  </si>
+  <si>
+    <t>લક્ષ્મણરાવ – પરશુરામપંત – પાંડુરંગપંત – વૈજનાથ –પાંડુરંગશાસ્ત્રી</t>
+  </si>
+  <si>
+    <t>લક્ષ્મણરાવ – પાંડુરંગપંત – પરશુરામપંત – વૈજનાથ –પાંડુરંગશાસ્ત્રી</t>
+  </si>
+  <si>
+    <t xml:space="preserve">દાદાજીએ આગરી લોકોને આપેલો પ્રયોગ </t>
+  </si>
+  <si>
+    <t>એકવીરા</t>
+  </si>
+  <si>
+    <t>ઘરમંદિર</t>
+  </si>
+  <si>
+    <t xml:space="preserve">મારા દીદી બતાવે જે રીતે.... ' આ ભાવગીત કઈ કેસેટમાં છે? </t>
+  </si>
+  <si>
+    <t>ન ત્વયા વિના</t>
+  </si>
+  <si>
+    <t>અશીતિ</t>
+  </si>
+  <si>
+    <t>તેજમિદમ્</t>
+  </si>
+  <si>
+    <t>નમઃ તે</t>
+  </si>
+  <si>
+    <t>ગણપતિના ઉત્સવને સામાજિક રૂપ આપનાર કોણ? </t>
+  </si>
+  <si>
+    <t>લોકમાન્ય તિલક</t>
+  </si>
+  <si>
+    <t>લાલા લજપતરાય</t>
+  </si>
+  <si>
+    <t>વીર સાવરકર</t>
+  </si>
+  <si>
+    <t>દયાનંદ સરસ્વતી</t>
+  </si>
+  <si>
+    <t>શ્રીરામરક્ષાસ્તોત્ર ના રચયિતા કોણ છે?</t>
+  </si>
+  <si>
+    <t>બુદ્ધકૌશિકમુનિ</t>
+  </si>
+  <si>
+    <t>ખંડનખંડખાદ્ય ગ્રંથના રચયિતા કોણ?</t>
+  </si>
+  <si>
+    <t>કાલિદાસ</t>
+  </si>
+  <si>
+    <t>ભવભૂતિ</t>
+  </si>
+  <si>
+    <t>ગુણાઢ્ય</t>
+  </si>
+  <si>
+    <t xml:space="preserve">સાત લાખ શ્લોક ધરાવતો પૈશાચી ભાષામાં લખાયેલ ગ્રંથ ના રચયિતા કોણ? </t>
+  </si>
+  <si>
+    <t>જીવનમાં કૃતજ્ઞતા નિર્માણ થાય એ માટે દાદાજીએ કઈ વાત આપી? </t>
+  </si>
+  <si>
+    <t>ભાવફેરી</t>
+  </si>
+  <si>
+    <t>ભક્તિફેરી</t>
+  </si>
+  <si>
+    <t>ત્રિકાળ સંધ્યા</t>
+  </si>
+  <si>
+    <t xml:space="preserve">વાચસ્પતિ મિશ્ર એ રચેલ ગ્રંથનું નામ </t>
+  </si>
+  <si>
+    <t>ખંડનખંડખાદ્ય</t>
+  </si>
+  <si>
+    <t>નૈષધ</t>
+  </si>
+  <si>
+    <t>ભામતી</t>
+  </si>
+  <si>
+    <t xml:space="preserve">યુવાકેન્દ્રની શરૂઆત કઈ સાલમાં થઇ? </t>
+  </si>
+  <si>
+    <t>વિદ્યાપ્રેમવર્ધન પરીક્ષાની શરૂઆત ક્યારથી થઈ?</t>
+  </si>
+  <si>
+    <t>સ્વાધ્યાય પરિવાર ના જિલ્લાના મુખ્ય કાર્યાલયને શું કહીએ છીએ?</t>
+  </si>
+  <si>
+    <t>નિર્મળ નિકેતન</t>
+  </si>
+  <si>
+    <t>વિમલ જ્યોતિ</t>
+  </si>
+  <si>
+    <t>પાર્થપ્રીતિ</t>
+  </si>
+  <si>
+    <t>આમાંથી એક પણ નહિ</t>
+  </si>
+  <si>
+    <t>ભાગવત પુરાણ માં કેટલા શ્લોકો છે?</t>
+  </si>
+  <si>
+    <t>નચિકેતા નું વર્ણન ક્યાં ઉપનિષદમાં આવે છે?</t>
+  </si>
+  <si>
+    <t>કેનોપનિષદ</t>
+  </si>
+  <si>
+    <t>ઈશાવાશ્યોપનીષદ</t>
+  </si>
+  <si>
+    <t>પ્રશ્નોપનિષદ</t>
+  </si>
+  <si>
+    <t>કઠોપનિષદ્</t>
+  </si>
+  <si>
+    <t>સાંદિપની ઋષિનો આશ્રમ કઈ નદીના કિનારે હતો?</t>
+  </si>
+  <si>
+    <t>કાવેરી</t>
+  </si>
+  <si>
+    <t>ક્ષિપ્રા</t>
+  </si>
+  <si>
+    <t>ગંગા</t>
+  </si>
+  <si>
+    <t>ભીષ્મપિતામહનુ મૂળ નામ</t>
+  </si>
+  <si>
+    <t>દેવવ્રત</t>
+  </si>
+  <si>
+    <t>રાધેય</t>
+  </si>
+  <si>
+    <t>દેવરત</t>
+  </si>
+  <si>
+    <t>દેવદત્ત</t>
+  </si>
+  <si>
+    <t>અભિમન્યુ ની પત્નીનું નામ</t>
+  </si>
+  <si>
+    <t>ઉત્તરા</t>
+  </si>
+  <si>
+    <t>ઊર્મિ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">કૃષ્ણના સારથી નું નામ </t>
+  </si>
+  <si>
+    <t>શલ્ય</t>
+  </si>
+  <si>
+    <t>ધૃષ્ટધ્રુમ્ન</t>
+  </si>
+  <si>
+    <t>વિરાટ</t>
+  </si>
+  <si>
+    <t>દારૂક</t>
+  </si>
+  <si>
+    <t xml:space="preserve">પ્લેટોના ગુરુ </t>
+  </si>
+  <si>
+    <t>કાર્લ માર્ક્સ</t>
+  </si>
+  <si>
+    <t>સોક્રેટિસ</t>
+  </si>
+  <si>
+    <t>જોહન આર્ક</t>
+  </si>
+  <si>
+    <t>ઈમર્સન</t>
+  </si>
+  <si>
+    <t xml:space="preserve">નવધા ભક્તિમાં બીજી ભક્તિ કઈ આવે છે? </t>
+  </si>
+  <si>
+    <t>कीर्तनम्</t>
+  </si>
+  <si>
+    <t xml:space="preserve">श्रवणम् </t>
+  </si>
+  <si>
+    <t xml:space="preserve">पादसेवनम् </t>
+  </si>
+  <si>
+    <t>सख्यम्</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ત્રિકાળ સંધ્યામાં ગીતાજીના શ્લોક કેટલા છે? </t>
+  </si>
+  <si>
+    <t>સ્વાધ્યાય પરિવારના કાર્યક્રમોમાં રાખવામાં આવતી પ્રાસંગિક ઓફિસ એટલે</t>
+  </si>
+  <si>
+    <t xml:space="preserve">યાતા યાત કાર્યાલય </t>
+  </si>
+  <si>
+    <t xml:space="preserve">પતંજલિ ચિકિત્સાલય </t>
+  </si>
+  <si>
+    <t>સુદામપુરી</t>
+  </si>
+  <si>
+    <t xml:space="preserve">અર્જુન કાર્યાલય </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ભીમના પૌત્ર નું નામ </t>
+  </si>
+  <si>
+    <t>ઘટોત્ઘચ</t>
+  </si>
+  <si>
+    <t>બર્બરીક</t>
+  </si>
+  <si>
+    <t>પરીક્ષિત</t>
+  </si>
+  <si>
+    <t>વિધાપીઠની સ્થાપના કયા વર્ષમાં થઇ?</t>
+  </si>
+  <si>
+    <t>વિદેશમાં સ્વાધ્યાય કાર્ય ક્યાં નામથી ચાલે છે?</t>
+  </si>
+  <si>
+    <t>Devine Association of Yogeshwar</t>
+  </si>
+  <si>
+    <t>Swadhyay Organization</t>
+  </si>
+  <si>
+    <t>Devine Society of Yogeshwar</t>
+  </si>
+  <si>
+    <t>Swadhyay Devine Family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">જીવનતીર્થ </t>
+  </si>
+  <si>
+    <t>hard</t>
+  </si>
+  <si>
+    <t>easy</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
 </sst>
 </file>
 
@@ -1135,7 +1657,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="[$-7000447]0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1176,6 +1698,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1210,7 +1745,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1248,6 +1783,16 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1530,7 +2075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I124"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="101.5703125" bestFit="1" customWidth="1"/>
@@ -3555,6 +4100,1164 @@
         <v>175</v>
       </c>
     </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="C77" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="D77" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="E77" s="18"/>
+      <c r="F77" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="G77" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="H77" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="B78" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="C78" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="D78" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="E78" s="18"/>
+      <c r="F78" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="G78" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="H78" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="B79" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="C79" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D79" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="E79" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="F79" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G79" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="H79" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="B80" s="18" t="s">
+        <v>366</v>
+      </c>
+      <c r="C80" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="D80" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="E80" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="F80" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="G80" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="H80" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="B81" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C81" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D81" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="E81" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="F81" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="G81" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="H81" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="B82" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="C82" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="D82" s="18" t="s">
+        <v>374</v>
+      </c>
+      <c r="E82" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="F82" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="G82" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="H82" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="18" t="s">
+        <v>376</v>
+      </c>
+      <c r="B83" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="C83" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D83" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="E83" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="F83" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="G83" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="H83" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="B84" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="C84" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D84" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="E84" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F84" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="G84" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="H84" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="18" t="s">
+        <v>383</v>
+      </c>
+      <c r="B85" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="C85" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="D85" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="E85" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="F85" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="G85" s="21" t="s">
+        <v>525</v>
+      </c>
+      <c r="H85" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" s="18" t="s">
+        <v>387</v>
+      </c>
+      <c r="B86" s="18">
+        <v>1995</v>
+      </c>
+      <c r="C86" s="18">
+        <v>1996</v>
+      </c>
+      <c r="D86" s="18">
+        <v>1997</v>
+      </c>
+      <c r="E86" s="18">
+        <v>1998</v>
+      </c>
+      <c r="F86" s="18">
+        <v>1997</v>
+      </c>
+      <c r="G86" s="18"/>
+      <c r="H86" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="B87" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="C87" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="D87" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="E87" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="F87" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="G87" s="18"/>
+      <c r="H87" s="18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="B88" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="C88" s="18" t="s">
+        <v>395</v>
+      </c>
+      <c r="D88" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="E88" s="18" t="s">
+        <v>397</v>
+      </c>
+      <c r="F88" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="G88" s="18"/>
+      <c r="H88" s="18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="18" t="s">
+        <v>398</v>
+      </c>
+      <c r="B89" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="C89" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="D89" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="E89" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="F89" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="G89" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="H89" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="B90" s="18" t="s">
+        <v>401</v>
+      </c>
+      <c r="C90" s="18" t="s">
+        <v>402</v>
+      </c>
+      <c r="D90" s="18" t="s">
+        <v>403</v>
+      </c>
+      <c r="E90" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="F90" s="18" t="s">
+        <v>401</v>
+      </c>
+      <c r="G90" s="18"/>
+      <c r="H90" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" s="18" t="s">
+        <v>405</v>
+      </c>
+      <c r="B91" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="C91" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="D91" s="18" t="s">
+        <v>408</v>
+      </c>
+      <c r="E91" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="F91" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="G91" s="18"/>
+      <c r="H91" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="18" t="s">
+        <v>410</v>
+      </c>
+      <c r="B92" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="C92" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="D92" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="E92" s="18" t="s">
+        <v>414</v>
+      </c>
+      <c r="F92" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G92" s="18"/>
+      <c r="H92" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="18" t="s">
+        <v>415</v>
+      </c>
+      <c r="B93" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="C93" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="D93" s="18" t="s">
+        <v>417</v>
+      </c>
+      <c r="E93" s="18" t="s">
+        <v>418</v>
+      </c>
+      <c r="F93" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="G93" s="18"/>
+      <c r="H93" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="B94" s="18" t="s">
+        <v>420</v>
+      </c>
+      <c r="C94" s="18" t="s">
+        <v>421</v>
+      </c>
+      <c r="D94" s="18"/>
+      <c r="E94" s="18"/>
+      <c r="F94" s="18"/>
+      <c r="G94" s="18"/>
+      <c r="H94" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="18" t="s">
+        <v>422</v>
+      </c>
+      <c r="B95" s="18">
+        <v>23</v>
+      </c>
+      <c r="C95" s="18">
+        <v>22</v>
+      </c>
+      <c r="D95" s="18">
+        <v>21</v>
+      </c>
+      <c r="E95" s="18">
+        <v>24</v>
+      </c>
+      <c r="F95" s="18">
+        <v>24</v>
+      </c>
+      <c r="G95" s="18"/>
+      <c r="H95" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="19" t="s">
+        <v>423</v>
+      </c>
+      <c r="B96" s="18" t="s">
+        <v>424</v>
+      </c>
+      <c r="C96" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="D96" s="18" t="s">
+        <v>426</v>
+      </c>
+      <c r="E96" s="18" t="s">
+        <v>427</v>
+      </c>
+      <c r="F96" s="18" t="s">
+        <v>424</v>
+      </c>
+      <c r="G96" s="18"/>
+      <c r="H96" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" s="18" t="s">
+        <v>428</v>
+      </c>
+      <c r="B97" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="C97" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D97" s="18" t="s">
+        <v>397</v>
+      </c>
+      <c r="E97" s="18" t="s">
+        <v>430</v>
+      </c>
+      <c r="F97" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="G97" s="18"/>
+      <c r="H97" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="B98" s="18" t="s">
+        <v>432</v>
+      </c>
+      <c r="C98" s="18" t="s">
+        <v>433</v>
+      </c>
+      <c r="D98" s="18" t="s">
+        <v>434</v>
+      </c>
+      <c r="E98" s="18" t="s">
+        <v>435</v>
+      </c>
+      <c r="F98" s="18" t="s">
+        <v>432</v>
+      </c>
+      <c r="G98" s="18"/>
+      <c r="H98" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" s="18" t="s">
+        <v>436</v>
+      </c>
+      <c r="B99" s="18">
+        <v>1987</v>
+      </c>
+      <c r="C99" s="18">
+        <v>1988</v>
+      </c>
+      <c r="D99" s="18">
+        <v>1989</v>
+      </c>
+      <c r="E99" s="18">
+        <v>1990</v>
+      </c>
+      <c r="F99" s="18">
+        <v>1988</v>
+      </c>
+      <c r="G99" s="18"/>
+      <c r="H99" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="B100" s="18" t="s">
+        <v>438</v>
+      </c>
+      <c r="C100" s="18" t="s">
+        <v>439</v>
+      </c>
+      <c r="D100" s="18" t="s">
+        <v>440</v>
+      </c>
+      <c r="E100" s="18"/>
+      <c r="F100" s="18" t="s">
+        <v>438</v>
+      </c>
+      <c r="G100" s="18"/>
+      <c r="H100" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" s="18" t="s">
+        <v>441</v>
+      </c>
+      <c r="B101" s="18" t="s">
+        <v>442</v>
+      </c>
+      <c r="C101" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="D101" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="E101" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="F101" s="18" t="s">
+        <v>442</v>
+      </c>
+      <c r="G101" s="18"/>
+      <c r="H101" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102" s="20" t="s">
+        <v>444</v>
+      </c>
+      <c r="B102" s="18" t="s">
+        <v>445</v>
+      </c>
+      <c r="C102" s="18" t="s">
+        <v>446</v>
+      </c>
+      <c r="D102" s="18" t="s">
+        <v>447</v>
+      </c>
+      <c r="E102" s="18" t="s">
+        <v>448</v>
+      </c>
+      <c r="F102" s="18" t="s">
+        <v>447</v>
+      </c>
+      <c r="G102" s="18"/>
+      <c r="H102" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103" s="18" t="s">
+        <v>449</v>
+      </c>
+      <c r="B103" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C103" s="18" t="s">
+        <v>451</v>
+      </c>
+      <c r="D103" s="18" t="s">
+        <v>452</v>
+      </c>
+      <c r="E103" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="F103" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G103" s="18"/>
+      <c r="H103" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104" s="18" t="s">
+        <v>454</v>
+      </c>
+      <c r="B104" s="18" t="s">
+        <v>455</v>
+      </c>
+      <c r="C104" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="D104" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="E104" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="F104" s="18" t="s">
+        <v>455</v>
+      </c>
+      <c r="G104" s="18"/>
+      <c r="H104" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105" s="18" t="s">
+        <v>456</v>
+      </c>
+      <c r="B105" s="18" t="s">
+        <v>457</v>
+      </c>
+      <c r="C105" s="18" t="s">
+        <v>458</v>
+      </c>
+      <c r="D105" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="E105" s="18" t="s">
+        <v>459</v>
+      </c>
+      <c r="F105" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="G105" s="18"/>
+      <c r="H105" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106" s="18" t="s">
+        <v>460</v>
+      </c>
+      <c r="B106" s="18" t="s">
+        <v>457</v>
+      </c>
+      <c r="C106" s="18" t="s">
+        <v>459</v>
+      </c>
+      <c r="D106" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="E106" s="18" t="s">
+        <v>458</v>
+      </c>
+      <c r="F106" s="18" t="s">
+        <v>459</v>
+      </c>
+      <c r="G106" s="18"/>
+      <c r="H106" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" s="18" t="s">
+        <v>461</v>
+      </c>
+      <c r="B107" s="18" t="s">
+        <v>462</v>
+      </c>
+      <c r="C107" s="18" t="s">
+        <v>463</v>
+      </c>
+      <c r="D107" s="18" t="s">
+        <v>464</v>
+      </c>
+      <c r="E107" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F107" s="21" t="s">
+        <v>464</v>
+      </c>
+      <c r="G107" s="18"/>
+      <c r="H107" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" s="18" t="s">
+        <v>465</v>
+      </c>
+      <c r="B108" s="18" t="s">
+        <v>466</v>
+      </c>
+      <c r="C108" s="18" t="s">
+        <v>467</v>
+      </c>
+      <c r="D108" s="18" t="s">
+        <v>468</v>
+      </c>
+      <c r="E108" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F108" s="18" t="s">
+        <v>468</v>
+      </c>
+      <c r="G108" s="18"/>
+      <c r="H108" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="18" t="s">
+        <v>469</v>
+      </c>
+      <c r="B109" s="18">
+        <v>1980</v>
+      </c>
+      <c r="C109" s="18">
+        <v>1979</v>
+      </c>
+      <c r="D109" s="18">
+        <v>1978</v>
+      </c>
+      <c r="E109" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F109" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="G109" s="18"/>
+      <c r="H109" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" s="22" t="s">
+        <v>470</v>
+      </c>
+      <c r="B110" s="23">
+        <v>1965</v>
+      </c>
+      <c r="C110" s="23">
+        <v>1966</v>
+      </c>
+      <c r="D110" s="23">
+        <v>1967</v>
+      </c>
+      <c r="E110" s="23">
+        <v>1968</v>
+      </c>
+      <c r="F110" s="23">
+        <v>1967</v>
+      </c>
+      <c r="G110" s="18"/>
+      <c r="H110" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111" s="22" t="s">
+        <v>471</v>
+      </c>
+      <c r="B111" s="22" t="s">
+        <v>472</v>
+      </c>
+      <c r="C111" s="22" t="s">
+        <v>473</v>
+      </c>
+      <c r="D111" s="22" t="s">
+        <v>474</v>
+      </c>
+      <c r="E111" s="22" t="s">
+        <v>475</v>
+      </c>
+      <c r="F111" s="22" t="s">
+        <v>474</v>
+      </c>
+      <c r="G111" s="18"/>
+      <c r="H111" s="22" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112" s="22" t="s">
+        <v>476</v>
+      </c>
+      <c r="B112" s="23">
+        <v>14500</v>
+      </c>
+      <c r="C112" s="23">
+        <v>14600</v>
+      </c>
+      <c r="D112" s="23">
+        <v>13500</v>
+      </c>
+      <c r="E112" s="23">
+        <v>13600</v>
+      </c>
+      <c r="F112" s="23">
+        <v>14500</v>
+      </c>
+      <c r="G112" s="18"/>
+      <c r="H112" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A113" s="22" t="s">
+        <v>477</v>
+      </c>
+      <c r="B113" s="22" t="s">
+        <v>478</v>
+      </c>
+      <c r="C113" s="22" t="s">
+        <v>479</v>
+      </c>
+      <c r="D113" s="22" t="s">
+        <v>480</v>
+      </c>
+      <c r="E113" s="22" t="s">
+        <v>481</v>
+      </c>
+      <c r="F113" s="22" t="s">
+        <v>481</v>
+      </c>
+      <c r="G113" s="18"/>
+      <c r="H113" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114" s="22" t="s">
+        <v>482</v>
+      </c>
+      <c r="B114" s="22" t="s">
+        <v>483</v>
+      </c>
+      <c r="C114" s="22" t="s">
+        <v>484</v>
+      </c>
+      <c r="D114" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E114" s="22" t="s">
+        <v>485</v>
+      </c>
+      <c r="F114" s="22" t="s">
+        <v>484</v>
+      </c>
+      <c r="G114" s="18"/>
+      <c r="H114" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115" s="22" t="s">
+        <v>486</v>
+      </c>
+      <c r="B115" s="22" t="s">
+        <v>487</v>
+      </c>
+      <c r="C115" s="22" t="s">
+        <v>488</v>
+      </c>
+      <c r="D115" s="22" t="s">
+        <v>489</v>
+      </c>
+      <c r="E115" s="22" t="s">
+        <v>490</v>
+      </c>
+      <c r="F115" s="22" t="s">
+        <v>487</v>
+      </c>
+      <c r="G115" s="18"/>
+      <c r="H115" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116" s="22" t="s">
+        <v>491</v>
+      </c>
+      <c r="B116" s="22" t="s">
+        <v>492</v>
+      </c>
+      <c r="C116" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="D116" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="E116" s="22" t="s">
+        <v>493</v>
+      </c>
+      <c r="F116" s="22" t="s">
+        <v>492</v>
+      </c>
+      <c r="G116" s="18"/>
+      <c r="H116" s="22" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117" s="22" t="s">
+        <v>494</v>
+      </c>
+      <c r="B117" s="22" t="s">
+        <v>495</v>
+      </c>
+      <c r="C117" s="22" t="s">
+        <v>496</v>
+      </c>
+      <c r="D117" s="22" t="s">
+        <v>497</v>
+      </c>
+      <c r="E117" s="22" t="s">
+        <v>498</v>
+      </c>
+      <c r="F117" s="22" t="s">
+        <v>498</v>
+      </c>
+      <c r="G117" s="18"/>
+      <c r="H117" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118" s="22" t="s">
+        <v>499</v>
+      </c>
+      <c r="B118" s="22" t="s">
+        <v>500</v>
+      </c>
+      <c r="C118" s="22" t="s">
+        <v>501</v>
+      </c>
+      <c r="D118" s="22" t="s">
+        <v>502</v>
+      </c>
+      <c r="E118" s="22" t="s">
+        <v>503</v>
+      </c>
+      <c r="F118" s="22" t="s">
+        <v>501</v>
+      </c>
+      <c r="G118" s="18"/>
+      <c r="H118" s="22" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119" s="22" t="s">
+        <v>504</v>
+      </c>
+      <c r="B119" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="C119" s="22" t="s">
+        <v>506</v>
+      </c>
+      <c r="D119" s="22" t="s">
+        <v>507</v>
+      </c>
+      <c r="E119" s="22" t="s">
+        <v>508</v>
+      </c>
+      <c r="F119" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="G119" s="18"/>
+      <c r="H119" s="22" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120" s="22" t="s">
+        <v>509</v>
+      </c>
+      <c r="B120" s="23">
+        <v>2</v>
+      </c>
+      <c r="C120" s="23">
+        <v>3</v>
+      </c>
+      <c r="D120" s="23">
+        <v>4</v>
+      </c>
+      <c r="E120" s="23">
+        <v>5</v>
+      </c>
+      <c r="F120" s="23">
+        <v>3</v>
+      </c>
+      <c r="G120" s="18"/>
+      <c r="H120" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121" s="22" t="s">
+        <v>510</v>
+      </c>
+      <c r="B121" s="22" t="s">
+        <v>511</v>
+      </c>
+      <c r="C121" s="22" t="s">
+        <v>512</v>
+      </c>
+      <c r="D121" s="22" t="s">
+        <v>513</v>
+      </c>
+      <c r="E121" s="22" t="s">
+        <v>514</v>
+      </c>
+      <c r="F121" s="22" t="s">
+        <v>514</v>
+      </c>
+      <c r="G121" s="18"/>
+      <c r="H121" s="22" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" s="22" t="s">
+        <v>515</v>
+      </c>
+      <c r="B122" s="22" t="s">
+        <v>516</v>
+      </c>
+      <c r="C122" s="22" t="s">
+        <v>517</v>
+      </c>
+      <c r="D122" s="22" t="s">
+        <v>518</v>
+      </c>
+      <c r="E122" s="22"/>
+      <c r="F122" s="22" t="s">
+        <v>517</v>
+      </c>
+      <c r="G122" s="18"/>
+      <c r="H122" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123" s="22" t="s">
+        <v>519</v>
+      </c>
+      <c r="B123" s="23">
+        <v>1926</v>
+      </c>
+      <c r="C123" s="23">
+        <v>1927</v>
+      </c>
+      <c r="D123" s="23">
+        <v>1956</v>
+      </c>
+      <c r="E123" s="23">
+        <v>1954</v>
+      </c>
+      <c r="F123" s="23">
+        <v>1956</v>
+      </c>
+      <c r="G123" s="18"/>
+      <c r="H123" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A124" s="22" t="s">
+        <v>520</v>
+      </c>
+      <c r="B124" s="22" t="s">
+        <v>521</v>
+      </c>
+      <c r="C124" s="22" t="s">
+        <v>522</v>
+      </c>
+      <c r="D124" s="22" t="s">
+        <v>523</v>
+      </c>
+      <c r="E124" s="22" t="s">
+        <v>524</v>
+      </c>
+      <c r="F124" s="22" t="s">
+        <v>521</v>
+      </c>
+      <c r="G124" s="18"/>
+      <c r="H124" s="22" t="s">
+        <v>526</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I76"/>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>